<commit_message>
Compare attributed Steam player and Metacritic critic ratings for PC deals
Replit-Task-Id: f98faccb-e7ac-4d1f-9ed2-432d7ee08535
Replit-Merge-Attempt: MergeTask:f98faccb-e7ac-4d1f-9ed2-432d7ee08535:1:3b53118f
</commit_message>
<xml_diff>
--- a/artifacts/api-server/data/game-deals.xlsx
+++ b/artifacts/api-server/data/game-deals.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="228">
   <si>
     <t>Steam App ID</t>
   </si>
@@ -38,6 +38,12 @@
     <t>Steam review count</t>
   </si>
   <si>
+    <t>Metacritic critic score (/100)</t>
+  </si>
+  <si>
+    <t>Metacritic link</t>
+  </si>
+  <si>
     <t>Dope score</t>
   </si>
   <si>
@@ -68,6 +74,9 @@
     <t>Action | Adventure</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/styx-shards-of-darkness?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=7bqsm2KowBN%2BhsqC1rikUJGjWUOSaGKQDYFAdr8cb8g%3D</t>
   </si>
   <si>
@@ -86,7 +95,7 @@
     <t>CheapShark / Steam</t>
   </si>
   <si>
-    <t>2026-09-26T07:26:17.183Z</t>
+    <t>2026-09-26T07:37:33.477Z</t>
   </si>
   <si>
     <t>A Fistful of Gun</t>
@@ -95,6 +104,9 @@
     <t>Action | Indie</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/a-fistful-of-gun?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=jI%2B9pViLtXA5z5SgIzhX6QtXR4G4DQn8OiqR1BFf8K4%3D</t>
   </si>
   <si>
@@ -113,6 +125,9 @@
     <t>Adventure</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/lost-horizon?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=lAzokTUYt5fAw5I9Lq9BNmS%2F%2FVmZ%2BZuCh%2FdjiUPhMCE%3D</t>
   </si>
   <si>
@@ -131,6 +146,9 @@
     <t>Adventure | Strategy</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/the-witcher-adventure-game?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=MxLPz2HWHmYzmNJnSvpw%2BPEadDhyPjjapZyi7rkTdBE%3D</t>
   </si>
   <si>
@@ -149,6 +167,9 @@
     <t>Adventure | Indie | RPG</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/winds-of-change?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=FgJB58yTlOi0r0ls3yNoipXcmbnXSRLpkDRiK7dyqRo%3D</t>
   </si>
   <si>
@@ -167,6 +188,9 @@
     <t>Action | RPG</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/deus-ex-human-revolution---directors-cut?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=HhzMJAgQYGZ%2B%2BFPpBG%2BRFcuUQZJO3KXvlnyYYGwGUfU%3D</t>
   </si>
   <si>
@@ -185,6 +209,9 @@
     <t>Action | Adventure | Indie</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=BGDNRb4tnJF6XR1JpxcgJIyM7RB3f9OHXzwhkH80ZsA%3D</t>
   </si>
   <si>
@@ -221,6 +248,9 @@
     <t>Indie | Racing</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/inertial-drift?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=NgBMsuyXzS0ro6GI4L%2B0mxrQbZ3o%2BkNsOlD4Un%2BWfMs%3D</t>
   </si>
   <si>
@@ -269,6 +299,9 @@
     <t>Action</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/ori-and-the-will-of-the-wisps?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=cOZmIEjtHzMQo8aqwzYPZvrEN%2BKt2as61wN%2FqbdxBJc%3D</t>
   </si>
   <si>
@@ -287,6 +320,9 @@
     <t>Action | Casual | Indie | Racing</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/speedrunners?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=9OGEXBHOruKD%2FmyCV5vggPcD6XSzaR1N5nNbd5%2FZrVg%3D</t>
   </si>
   <si>
@@ -302,6 +338,9 @@
     <t>Sanctum 2</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/sanctum-2?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=yZOw9npDUh1Qvb%2FPw24dTNy5ruNIL8q1kK3fl2lwNWM%3D</t>
   </si>
   <si>
@@ -356,6 +395,9 @@
     <t>Racing | Simulation | Sports</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/wrc-8-fia-world-rally-championship?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=8XDw%2FS456jlKkVNjgE%2FacR3voVCFNrEAH%2FipVFLnu1Q%3D</t>
   </si>
   <si>
@@ -371,6 +413,9 @@
     <t>Deus Ex: Mankind Divided</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/deus-ex-mankind-divided?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=Ppi1hduzzSTTcVfyap53KkMwyHbwS8In80ZKCDLt3I4%3D</t>
   </si>
   <si>
@@ -404,6 +449,9 @@
     <t>Rogue Stormers</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/rogue-stormers?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=TXFZalGoZbJ6Mi8m%2FcQKbvwebSAE5tmBnIuw3JhvhLE%3D</t>
   </si>
   <si>
@@ -422,6 +470,9 @@
     <t>Adventure | RPG</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/thronebreaker-the-witcher-tales?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=MXSExE9i1D1PUieET9Zp7CGZGgZ62GDvffKyV9gsWOE%3D</t>
   </si>
   <si>
@@ -437,6 +488,9 @@
     <t>Borderlands: The Pre-Sequel</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/borderlands-the-pre-sequel?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=MMTKpgFFpjanMzaUVCze4ETCgy6FtTebuJZfYUptveQ%3D</t>
   </si>
   <si>
@@ -455,6 +509,9 @@
     <t>Simulation</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/hypnospace-outlaw?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=mP5QNP2xVSeJYUfkVf403hN9ZPSvI1nYCYy3a27r%2B4w%3D</t>
   </si>
   <si>
@@ -470,6 +527,9 @@
     <t>Ori and the Blind Forest: Definitive Edition</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/ori-and-the-blind-forest-definitive-edition?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=5FvRYOyTI%2BDQ1gtsb9zR8kwkz39p0HZrAqegVciljA0%3D</t>
   </si>
   <si>
@@ -485,6 +545,9 @@
     <t>Borderlands 2</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/borderlands-2?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=y9vH5Xf2O3lmQzX8IprLnYJ8PT7C2MafD4gPIMz7y%2Fs%3D</t>
   </si>
   <si>
@@ -503,6 +566,9 @@
     <t>Action | Indie | RPG</t>
   </si>
   <si>
+    <t>https://www.metacritic.com/game/pc/hades?ftag=MCD-06-10aaa1f</t>
+  </si>
+  <si>
     <t>https://www.cheapshark.com/redirect?dealID=%2FRRvRbW4trH2Me4HcfUIFk5pCGamwlMuyid9ZTDJ4do%3D</t>
   </si>
   <si>
@@ -597,6 +663,12 @@
   </si>
   <si>
     <t>CheapShark's Steam positive-review percentage, converted to a 5-point scale</t>
+  </si>
+  <si>
+    <t>Optional critic rating</t>
+  </si>
+  <si>
+    <t>Metacritic PC critic score and link supplied by Steam game details; 0–100 divided by 20 for display only, not included in the Dope score.</t>
   </si>
   <si>
     <t>(Discount percentage points × Steam rating out of 5) ÷ sale price in USD</t>
@@ -1039,7 +1111,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:R30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1049,17 +1121,19 @@
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
     <col min="7" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="48" customWidth="1"/>
-    <col min="11" max="11" width="46" customWidth="1"/>
-    <col min="12" max="12" width="49" customWidth="1"/>
-    <col min="13" max="13" width="58" customWidth="1"/>
-    <col min="14" max="14" width="16" customWidth="1"/>
-    <col min="15" max="15" width="18" customWidth="1"/>
-    <col min="16" max="16" width="27" customWidth="1"/>
+    <col min="9" max="9" width="28" customWidth="1"/>
+    <col min="10" max="10" width="54" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="48" customWidth="1"/>
+    <col min="13" max="13" width="46" customWidth="1"/>
+    <col min="14" max="14" width="49" customWidth="1"/>
+    <col min="15" max="15" width="58" customWidth="1"/>
+    <col min="16" max="16" width="16" customWidth="1"/>
+    <col min="17" max="17" width="18" customWidth="1"/>
+    <col min="18" max="18" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1108,16 +1182,22 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>355790</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D2" s="2">
         <v>1.39</v>
@@ -1134,41 +1214,47 @@
       <c r="H2">
         <v>2252</v>
       </c>
-      <c r="I2" s="3">
+      <c r="I2">
+        <v>72</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="3">
         <f>IFERROR(F2*G2/D2,0)</f>
         <v>277.66</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>19</v>
-      </c>
       <c r="L2" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="M2" t="s">
         <v>21</v>
       </c>
-      <c r="N2" t="s">
+      <c r="M2" s="4" t="s">
         <v>22</v>
       </c>
+      <c r="N2" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="O2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>26</v>
+      </c>
+      <c r="R2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>229810</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D3" s="6">
         <v>0.99</v>
@@ -1185,41 +1271,47 @@
       <c r="H3" s="5">
         <v>137</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="5">
+        <v>60</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" s="7">
         <f>IFERROR(F3*G3/D3,0)</f>
         <v>268.18</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="L3" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="K3" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="L3" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="P3" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>40350</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D4" s="2">
         <v>1.49</v>
@@ -1236,41 +1328,47 @@
       <c r="H4">
         <v>460</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4">
+        <v>77</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="K4" s="3">
         <f>IFERROR(F4*G4/D4,0)</f>
         <v>259.56</v>
       </c>
-      <c r="J4" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>34</v>
-      </c>
       <c r="L4" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="M4" t="s">
-        <v>36</v>
-      </c>
-      <c r="N4" t="s">
-        <v>22</v>
+        <v>38</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="O4" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="P4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>26</v>
+      </c>
+      <c r="R4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>303800</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D5" s="6">
         <v>1.49</v>
@@ -1287,41 +1385,47 @@
       <c r="H5" s="5">
         <v>1178</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="5">
+        <v>68</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="K5" s="7">
         <f>IFERROR(F5*G5/D5,0)</f>
         <v>219.63</v>
       </c>
-      <c r="J5" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="K5" s="8" t="s">
-        <v>40</v>
-      </c>
       <c r="L5" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="M5" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>22</v>
+        <v>45</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="N5" s="8" t="s">
+        <v>47</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="P5" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R5" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>594130</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D6" s="2">
         <v>1.99</v>
@@ -1338,41 +1442,47 @@
       <c r="H6">
         <v>551</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I6">
+        <v>74</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="K6" s="3">
         <f>IFERROR(F6*G6/D6,0)</f>
         <v>214.82</v>
       </c>
-      <c r="J6" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>46</v>
-      </c>
       <c r="L6" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="M6" t="s">
-        <v>48</v>
-      </c>
-      <c r="N6" t="s">
-        <v>22</v>
+        <v>52</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="O6" t="s">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="P6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>26</v>
+      </c>
+      <c r="R6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>238010</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D7" s="6">
         <v>1.99</v>
@@ -1389,41 +1499,47 @@
       <c r="H7" s="5">
         <v>13552</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="5">
+        <v>91</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="K7" s="7">
         <f>IFERROR(F7*G7/D7,0)</f>
         <v>205.78</v>
       </c>
-      <c r="J7" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="K7" s="8" t="s">
-        <v>52</v>
-      </c>
       <c r="L7" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="M7" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="N7" s="5" t="s">
-        <v>22</v>
+        <v>59</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="N7" s="8" t="s">
+        <v>61</v>
       </c>
       <c r="O7" s="5" t="s">
-        <v>23</v>
+        <v>62</v>
       </c>
       <c r="P7" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R7" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>653060</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="C8" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D8" s="2">
         <v>1.49</v>
@@ -1440,41 +1556,47 @@
       <c r="H8">
         <v>181</v>
       </c>
-      <c r="I8" s="3">
+      <c r="I8" t="s">
+        <v>65</v>
+      </c>
+      <c r="J8" t="s">
+        <v>65</v>
+      </c>
+      <c r="K8" s="3">
         <f>IFERROR(F8*G8/D8,0)</f>
         <v>193.29</v>
       </c>
-      <c r="J8" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="L8" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="M8" t="s">
-        <v>60</v>
-      </c>
-      <c r="N8" t="s">
-        <v>22</v>
+        <v>66</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>68</v>
       </c>
       <c r="O8" t="s">
-        <v>23</v>
+        <v>69</v>
       </c>
       <c r="P8" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>26</v>
+      </c>
+      <c r="R8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>820520</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="D9" s="6">
         <v>1.99</v>
@@ -1491,41 +1613,47 @@
       <c r="H9" s="5">
         <v>3710</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="K9" s="7">
         <f>IFERROR(F9*G9/D9,0)</f>
         <v>189.95</v>
       </c>
-      <c r="J9" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>64</v>
-      </c>
       <c r="L9" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="M9" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="N9" s="5" t="s">
-        <v>22</v>
+        <v>72</v>
+      </c>
+      <c r="M9" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="N9" s="8" t="s">
+        <v>74</v>
       </c>
       <c r="O9" s="5" t="s">
-        <v>23</v>
+        <v>75</v>
       </c>
       <c r="P9" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R9" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1184480</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="C10" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="D10" s="2">
         <v>1.99</v>
@@ -1542,41 +1670,47 @@
       <c r="H10">
         <v>1329</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10">
+        <v>89</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="K10" s="3">
         <f>IFERROR(F10*G10/D10,0)</f>
         <v>189.95</v>
       </c>
-      <c r="J10" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>70</v>
-      </c>
       <c r="L10" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="M10" t="s">
-        <v>72</v>
-      </c>
-      <c r="N10" t="s">
-        <v>22</v>
+        <v>79</v>
+      </c>
+      <c r="M10" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="N10" s="4" t="s">
+        <v>81</v>
       </c>
       <c r="O10" t="s">
-        <v>23</v>
+        <v>82</v>
       </c>
       <c r="P10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>2161620</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="D11" s="6">
         <v>1.99</v>
@@ -1593,41 +1727,47 @@
       <c r="H11" s="5">
         <v>155</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="K11" s="7">
         <f>IFERROR(F11*G11/D11,0)</f>
         <v>165.08</v>
       </c>
-      <c r="J11" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="K11" s="8" t="s">
-        <v>75</v>
-      </c>
       <c r="L11" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="M11" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="N11" s="5" t="s">
-        <v>22</v>
+        <v>84</v>
+      </c>
+      <c r="M11" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="N11" s="8" t="s">
+        <v>86</v>
       </c>
       <c r="O11" s="5" t="s">
-        <v>23</v>
+        <v>87</v>
       </c>
       <c r="P11" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q11" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R11" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>773740</v>
       </c>
       <c r="B12" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C12" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="D12" s="2">
         <v>1.49</v>
@@ -1644,41 +1784,47 @@
       <c r="H12">
         <v>106</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" t="s">
+        <v>65</v>
+      </c>
+      <c r="J12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K12" s="3">
         <f>IFERROR(F12*G12/D12,0)</f>
         <v>159.4</v>
       </c>
-      <c r="J12" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>80</v>
-      </c>
       <c r="L12" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="M12" t="s">
-        <v>82</v>
-      </c>
-      <c r="N12" t="s">
-        <v>22</v>
+        <v>89</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="N12" s="4" t="s">
+        <v>91</v>
       </c>
       <c r="O12" t="s">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="P12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>26</v>
+      </c>
+      <c r="R12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>1057090</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="D13" s="6">
         <v>2.99</v>
@@ -1695,41 +1841,47 @@
       <c r="H13" s="5">
         <v>31214</v>
       </c>
-      <c r="I13" s="7">
+      <c r="I13" s="5">
+        <v>88</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="K13" s="7">
         <f>IFERROR(F13*G13/D13,0)</f>
         <v>144.48</v>
       </c>
-      <c r="J13" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="K13" s="8" t="s">
-        <v>86</v>
-      </c>
       <c r="L13" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="M13" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="N13" s="5" t="s">
-        <v>22</v>
+        <v>96</v>
+      </c>
+      <c r="M13" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="N13" s="8" t="s">
+        <v>98</v>
       </c>
       <c r="O13" s="5" t="s">
-        <v>23</v>
+        <v>99</v>
       </c>
       <c r="P13" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q13" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R13" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>207140</v>
       </c>
       <c r="B14" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="C14" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="D14" s="2">
         <v>2.99</v>
@@ -1746,41 +1898,47 @@
       <c r="H14">
         <v>9658</v>
       </c>
-      <c r="I14" s="3">
+      <c r="I14">
+        <v>84</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="K14" s="3">
         <f>IFERROR(F14*G14/D14,0)</f>
         <v>125.75</v>
       </c>
-      <c r="J14" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>92</v>
-      </c>
       <c r="L14" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="M14" t="s">
-        <v>94</v>
-      </c>
-      <c r="N14" t="s">
-        <v>22</v>
+        <v>103</v>
+      </c>
+      <c r="M14" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="N14" s="4" t="s">
+        <v>105</v>
       </c>
       <c r="O14" t="s">
-        <v>23</v>
+        <v>106</v>
       </c>
       <c r="P14" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>26</v>
+      </c>
+      <c r="R14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>210770</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="D15" s="6">
         <v>2.99</v>
@@ -1797,41 +1955,47 @@
       <c r="H15" s="5">
         <v>4345</v>
       </c>
-      <c r="I15" s="7">
+      <c r="I15" s="5">
+        <v>77</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="K15" s="7">
         <f>IFERROR(F15*G15/D15,0)</f>
         <v>123.08</v>
       </c>
-      <c r="J15" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="K15" s="8" t="s">
-        <v>97</v>
-      </c>
       <c r="L15" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="M15" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="N15" s="5" t="s">
-        <v>22</v>
+        <v>109</v>
+      </c>
+      <c r="M15" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="N15" s="8" t="s">
+        <v>111</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>23</v>
+        <v>112</v>
       </c>
       <c r="P15" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q15" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R15" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>1912380</v>
       </c>
       <c r="B16" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="C16" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="D16" s="2">
         <v>1.99</v>
@@ -1848,41 +2012,47 @@
       <c r="H16">
         <v>123</v>
       </c>
-      <c r="I16" s="3">
+      <c r="I16" t="s">
+        <v>65</v>
+      </c>
+      <c r="J16" t="s">
+        <v>65</v>
+      </c>
+      <c r="K16" s="3">
         <f>IFERROR(F16*G16/D16,0)</f>
         <v>119.85</v>
       </c>
-      <c r="J16" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="K16" s="4" t="s">
-        <v>103</v>
-      </c>
       <c r="L16" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="M16" t="s">
-        <v>105</v>
-      </c>
-      <c r="N16" t="s">
-        <v>22</v>
+        <v>115</v>
+      </c>
+      <c r="M16" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="N16" s="4" t="s">
+        <v>117</v>
       </c>
       <c r="O16" t="s">
-        <v>23</v>
+        <v>118</v>
       </c>
       <c r="P16" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>26</v>
+      </c>
+      <c r="R16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
         <v>1975440</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="D17" s="6">
         <v>2.99</v>
@@ -1899,41 +2069,47 @@
       <c r="H17" s="5">
         <v>1697</v>
       </c>
-      <c r="I17" s="7">
+      <c r="I17" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="K17" s="7">
         <f>IFERROR(F17*G17/D17,0)</f>
         <v>115.89</v>
       </c>
-      <c r="J17" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="K17" s="8" t="s">
-        <v>109</v>
-      </c>
       <c r="L17" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="M17" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="N17" s="5" t="s">
-        <v>22</v>
+        <v>121</v>
+      </c>
+      <c r="M17" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="N17" s="8" t="s">
+        <v>123</v>
       </c>
       <c r="O17" s="5" t="s">
-        <v>23</v>
+        <v>124</v>
       </c>
       <c r="P17" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q17" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R17" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>1004750</v>
       </c>
       <c r="B18" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="C18" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="D18" s="2">
         <v>2.99</v>
@@ -1950,41 +2126,47 @@
       <c r="H18">
         <v>427</v>
       </c>
-      <c r="I18" s="3">
+      <c r="I18">
+        <v>77</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="K18" s="3">
         <f>IFERROR(F18*G18/D18,0)</f>
         <v>115.89</v>
       </c>
-      <c r="J18" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="K18" s="4" t="s">
-        <v>115</v>
-      </c>
       <c r="L18" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="M18" t="s">
-        <v>117</v>
-      </c>
-      <c r="N18" t="s">
-        <v>22</v>
+        <v>128</v>
+      </c>
+      <c r="M18" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="N18" s="4" t="s">
+        <v>130</v>
       </c>
       <c r="O18" t="s">
-        <v>23</v>
+        <v>131</v>
       </c>
       <c r="P18" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>26</v>
+      </c>
+      <c r="R18" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>337000</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D19" s="6">
         <v>2.99</v>
@@ -2001,41 +2183,47 @@
       <c r="H19" s="5">
         <v>16490</v>
       </c>
-      <c r="I19" s="7">
+      <c r="I19" s="5">
+        <v>83</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="K19" s="7">
         <f>IFERROR(F19*G19/D19,0)</f>
         <v>112.88</v>
       </c>
-      <c r="J19" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="K19" s="8" t="s">
-        <v>120</v>
-      </c>
       <c r="L19" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="M19" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="N19" s="5" t="s">
-        <v>22</v>
+        <v>134</v>
+      </c>
+      <c r="M19" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="N19" s="8" t="s">
+        <v>136</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>23</v>
+        <v>137</v>
       </c>
       <c r="P19" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q19" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R19" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>921800</v>
       </c>
       <c r="B20" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="C20" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="D20" s="2">
         <v>2.99</v>
@@ -2052,41 +2240,47 @@
       <c r="H20">
         <v>2095</v>
       </c>
-      <c r="I20" s="3">
+      <c r="I20" t="s">
+        <v>65</v>
+      </c>
+      <c r="J20" t="s">
+        <v>65</v>
+      </c>
+      <c r="K20" s="3">
         <f>IFERROR(F20*G20/D20,0)</f>
         <v>111.37</v>
       </c>
-      <c r="J20" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="K20" s="4" t="s">
-        <v>126</v>
-      </c>
       <c r="L20" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="M20" t="s">
-        <v>128</v>
-      </c>
-      <c r="N20" t="s">
-        <v>22</v>
+        <v>140</v>
+      </c>
+      <c r="M20" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="N20" s="4" t="s">
+        <v>142</v>
       </c>
       <c r="O20" t="s">
-        <v>23</v>
+        <v>143</v>
       </c>
       <c r="P20" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>26</v>
+      </c>
+      <c r="R20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>299480</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D21" s="6">
         <v>2.99</v>
@@ -2103,41 +2297,47 @@
       <c r="H21" s="5">
         <v>650</v>
       </c>
-      <c r="I21" s="7">
+      <c r="I21" s="5">
+        <v>68</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="K21" s="7">
         <f>IFERROR(F21*G21/D21,0)</f>
         <v>92.39</v>
       </c>
-      <c r="J21" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="K21" s="8" t="s">
-        <v>131</v>
-      </c>
       <c r="L21" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="M21" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="N21" s="5" t="s">
-        <v>22</v>
+        <v>146</v>
+      </c>
+      <c r="M21" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="N21" s="8" t="s">
+        <v>148</v>
       </c>
       <c r="O21" s="5" t="s">
-        <v>23</v>
+        <v>149</v>
       </c>
       <c r="P21" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q21" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R21" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>973760</v>
       </c>
       <c r="B22" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="C22" t="s">
-        <v>135</v>
+        <v>151</v>
       </c>
       <c r="D22" s="2">
         <v>3.99</v>
@@ -2154,41 +2354,47 @@
       <c r="H22">
         <v>4721</v>
       </c>
-      <c r="I22" s="3">
+      <c r="I22">
+        <v>85</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="K22" s="3">
         <f>IFERROR(F22*G22/D22,0)</f>
         <v>87.22</v>
       </c>
-      <c r="J22" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="K22" s="4" t="s">
-        <v>137</v>
-      </c>
       <c r="L22" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="M22" t="s">
-        <v>139</v>
-      </c>
-      <c r="N22" t="s">
-        <v>22</v>
+        <v>153</v>
+      </c>
+      <c r="M22" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="N22" s="4" t="s">
+        <v>155</v>
       </c>
       <c r="O22" t="s">
-        <v>23</v>
+        <v>156</v>
       </c>
       <c r="P22" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>26</v>
+      </c>
+      <c r="R22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
         <v>261640</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D23" s="6">
         <v>3.99</v>
@@ -2205,41 +2411,47 @@
       <c r="H23" s="5">
         <v>19066</v>
       </c>
-      <c r="I23" s="7">
+      <c r="I23" s="5">
+        <v>75</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="K23" s="7">
         <f>IFERROR(F23*G23/D23,0)</f>
         <v>84.59</v>
       </c>
-      <c r="J23" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="K23" s="8" t="s">
-        <v>142</v>
-      </c>
       <c r="L23" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="M23" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="N23" s="5" t="s">
-        <v>22</v>
+        <v>159</v>
+      </c>
+      <c r="M23" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="N23" s="8" t="s">
+        <v>161</v>
       </c>
       <c r="O23" s="5" t="s">
-        <v>23</v>
+        <v>162</v>
       </c>
       <c r="P23" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q23" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R23" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>844590</v>
       </c>
       <c r="B24" t="s">
-        <v>145</v>
+        <v>163</v>
       </c>
       <c r="C24" t="s">
-        <v>146</v>
+        <v>164</v>
       </c>
       <c r="D24" s="2">
         <v>4.99</v>
@@ -2256,41 +2468,47 @@
       <c r="H24">
         <v>4389</v>
       </c>
-      <c r="I24" s="3">
+      <c r="I24">
+        <v>83</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="K24" s="3">
         <f>IFERROR(F24*G24/D24,0)</f>
         <v>72.14</v>
       </c>
-      <c r="J24" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="K24" s="4" t="s">
-        <v>148</v>
-      </c>
       <c r="L24" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="M24" t="s">
-        <v>150</v>
-      </c>
-      <c r="N24" t="s">
-        <v>22</v>
+        <v>166</v>
+      </c>
+      <c r="M24" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="N24" s="4" t="s">
+        <v>168</v>
       </c>
       <c r="O24" t="s">
-        <v>23</v>
+        <v>169</v>
       </c>
       <c r="P24" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>26</v>
+      </c>
+      <c r="R24" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
         <v>387290</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>151</v>
+        <v>170</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="D25" s="6">
         <v>4.99</v>
@@ -2307,41 +2525,47 @@
       <c r="H25" s="5">
         <v>30810</v>
       </c>
-      <c r="I25" s="7">
+      <c r="I25" s="5">
+        <v>88</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="K25" s="7">
         <f>IFERROR(F25*G25/D25,0)</f>
         <v>69.89</v>
       </c>
-      <c r="J25" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="K25" s="8" t="s">
-        <v>153</v>
-      </c>
       <c r="L25" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="M25" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="N25" s="5" t="s">
-        <v>22</v>
+        <v>172</v>
+      </c>
+      <c r="M25" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="N25" s="8" t="s">
+        <v>174</v>
       </c>
       <c r="O25" s="5" t="s">
-        <v>23</v>
+        <v>175</v>
       </c>
       <c r="P25" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q25" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R25" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>49520</v>
       </c>
       <c r="B26" t="s">
-        <v>156</v>
+        <v>176</v>
       </c>
       <c r="C26" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D26" s="2">
         <v>5.99</v>
@@ -2358,41 +2582,47 @@
       <c r="H26">
         <v>122931</v>
       </c>
-      <c r="I26" s="3">
+      <c r="I26">
+        <v>89</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="K26" s="3">
         <f>IFERROR(F26*G26/D26,0)</f>
         <v>63.86</v>
       </c>
-      <c r="J26" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="K26" s="4" t="s">
-        <v>158</v>
-      </c>
       <c r="L26" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="M26" t="s">
-        <v>160</v>
-      </c>
-      <c r="N26" t="s">
-        <v>22</v>
+        <v>178</v>
+      </c>
+      <c r="M26" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="N26" s="4" t="s">
+        <v>180</v>
       </c>
       <c r="O26" t="s">
-        <v>23</v>
+        <v>181</v>
       </c>
       <c r="P26" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>26</v>
+      </c>
+      <c r="R26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
         <v>1145360</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>162</v>
+        <v>183</v>
       </c>
       <c r="D27" s="6">
         <v>6.24</v>
@@ -2409,41 +2639,47 @@
       <c r="H27" s="5">
         <v>142544</v>
       </c>
-      <c r="I27" s="7">
+      <c r="I27" s="5">
+        <v>93</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>184</v>
+      </c>
+      <c r="K27" s="7">
         <f>IFERROR(F27*G27/D27,0)</f>
         <v>58.89</v>
       </c>
-      <c r="J27" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="K27" s="8" t="s">
-        <v>164</v>
-      </c>
       <c r="L27" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="M27" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="N27" s="5" t="s">
-        <v>22</v>
+        <v>185</v>
+      </c>
+      <c r="M27" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="N27" s="8" t="s">
+        <v>187</v>
       </c>
       <c r="O27" s="5" t="s">
-        <v>23</v>
+        <v>188</v>
       </c>
       <c r="P27" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q27" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R27" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>234080</v>
       </c>
       <c r="B28" t="s">
-        <v>167</v>
+        <v>189</v>
       </c>
       <c r="C28" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D28" s="2">
         <v>5.99</v>
@@ -2460,41 +2696,47 @@
       <c r="H28">
         <v>3228</v>
       </c>
-      <c r="I28" s="3">
+      <c r="I28" t="s">
+        <v>65</v>
+      </c>
+      <c r="J28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K28" s="3">
         <f>IFERROR(F28*G28/D28,0)</f>
         <v>48.08</v>
       </c>
-      <c r="J28" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="K28" s="4" t="s">
-        <v>169</v>
-      </c>
       <c r="L28" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="M28" t="s">
-        <v>171</v>
-      </c>
-      <c r="N28" t="s">
-        <v>22</v>
+        <v>190</v>
+      </c>
+      <c r="M28" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="N28" s="4" t="s">
+        <v>192</v>
       </c>
       <c r="O28" t="s">
-        <v>23</v>
+        <v>193</v>
       </c>
       <c r="P28" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>26</v>
+      </c>
+      <c r="R28" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
         <v>3407390</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>172</v>
+        <v>194</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>173</v>
+        <v>195</v>
       </c>
       <c r="D29" s="6">
         <v>24.99</v>
@@ -2511,41 +2753,47 @@
       <c r="H29" s="5">
         <v>1933</v>
       </c>
-      <c r="I29" s="7">
+      <c r="I29" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="K29" s="7">
         <f>IFERROR(F29*G29/D29,0)</f>
         <v>8.3</v>
       </c>
-      <c r="J29" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="K29" s="8" t="s">
-        <v>175</v>
-      </c>
       <c r="L29" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="M29" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="N29" s="5" t="s">
-        <v>22</v>
+        <v>196</v>
+      </c>
+      <c r="M29" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="N29" s="8" t="s">
+        <v>198</v>
       </c>
       <c r="O29" s="5" t="s">
-        <v>23</v>
+        <v>199</v>
       </c>
       <c r="P29" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="Q29" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R29" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>4358690</v>
       </c>
       <c r="B30" t="s">
-        <v>178</v>
+        <v>200</v>
       </c>
       <c r="C30" t="s">
-        <v>179</v>
+        <v>201</v>
       </c>
       <c r="D30" s="2">
         <v>23.18</v>
@@ -2562,122 +2810,147 @@
       <c r="H30">
         <v>1502</v>
       </c>
-      <c r="I30" s="3">
+      <c r="I30" t="s">
+        <v>65</v>
+      </c>
+      <c r="J30" t="s">
+        <v>65</v>
+      </c>
+      <c r="K30" s="3">
         <f>IFERROR(F30*G30/D30,0)</f>
         <v>6.68</v>
       </c>
-      <c r="J30" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="K30" s="4" t="s">
-        <v>181</v>
-      </c>
       <c r="L30" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="M30" t="s">
-        <v>183</v>
-      </c>
-      <c r="N30" t="s">
-        <v>22</v>
+        <v>202</v>
+      </c>
+      <c r="M30" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="N30" s="4" t="s">
+        <v>204</v>
       </c>
       <c r="O30" t="s">
-        <v>23</v>
+        <v>205</v>
       </c>
       <c r="P30" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>26</v>
+      </c>
+      <c r="R30" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P30"/>
+  <autoFilter ref="A1:R30"/>
   <hyperlinks>
     <hyperlink ref="J2" r:id="rId1"/>
-    <hyperlink ref="K2" r:id="rId2"/>
-    <hyperlink ref="L2" r:id="rId3"/>
-    <hyperlink ref="J3" r:id="rId4"/>
-    <hyperlink ref="K3" r:id="rId5"/>
+    <hyperlink ref="L2" r:id="rId2"/>
+    <hyperlink ref="M2" r:id="rId3"/>
+    <hyperlink ref="N2" r:id="rId4"/>
+    <hyperlink ref="J3" r:id="rId5"/>
     <hyperlink ref="L3" r:id="rId6"/>
-    <hyperlink ref="J4" r:id="rId7"/>
-    <hyperlink ref="K4" r:id="rId8"/>
-    <hyperlink ref="L4" r:id="rId9"/>
-    <hyperlink ref="J5" r:id="rId10"/>
-    <hyperlink ref="K5" r:id="rId11"/>
-    <hyperlink ref="L5" r:id="rId12"/>
-    <hyperlink ref="J6" r:id="rId13"/>
-    <hyperlink ref="K6" r:id="rId14"/>
-    <hyperlink ref="L6" r:id="rId15"/>
-    <hyperlink ref="J7" r:id="rId16"/>
-    <hyperlink ref="K7" r:id="rId17"/>
-    <hyperlink ref="L7" r:id="rId18"/>
-    <hyperlink ref="J8" r:id="rId19"/>
-    <hyperlink ref="K8" r:id="rId20"/>
-    <hyperlink ref="L8" r:id="rId21"/>
-    <hyperlink ref="J9" r:id="rId22"/>
-    <hyperlink ref="K9" r:id="rId23"/>
-    <hyperlink ref="L9" r:id="rId24"/>
-    <hyperlink ref="J10" r:id="rId25"/>
-    <hyperlink ref="K10" r:id="rId26"/>
-    <hyperlink ref="L10" r:id="rId27"/>
-    <hyperlink ref="J11" r:id="rId28"/>
-    <hyperlink ref="K11" r:id="rId29"/>
-    <hyperlink ref="L11" r:id="rId30"/>
-    <hyperlink ref="J12" r:id="rId31"/>
-    <hyperlink ref="K12" r:id="rId32"/>
-    <hyperlink ref="L12" r:id="rId33"/>
-    <hyperlink ref="J13" r:id="rId34"/>
-    <hyperlink ref="K13" r:id="rId35"/>
-    <hyperlink ref="L13" r:id="rId36"/>
-    <hyperlink ref="J14" r:id="rId37"/>
-    <hyperlink ref="K14" r:id="rId38"/>
-    <hyperlink ref="L14" r:id="rId39"/>
-    <hyperlink ref="J15" r:id="rId40"/>
-    <hyperlink ref="K15" r:id="rId41"/>
-    <hyperlink ref="L15" r:id="rId42"/>
-    <hyperlink ref="J16" r:id="rId43"/>
-    <hyperlink ref="K16" r:id="rId44"/>
-    <hyperlink ref="L16" r:id="rId45"/>
-    <hyperlink ref="J17" r:id="rId46"/>
-    <hyperlink ref="K17" r:id="rId47"/>
-    <hyperlink ref="L17" r:id="rId48"/>
-    <hyperlink ref="J18" r:id="rId49"/>
-    <hyperlink ref="K18" r:id="rId50"/>
-    <hyperlink ref="L18" r:id="rId51"/>
-    <hyperlink ref="J19" r:id="rId52"/>
-    <hyperlink ref="K19" r:id="rId53"/>
-    <hyperlink ref="L19" r:id="rId54"/>
-    <hyperlink ref="J20" r:id="rId55"/>
-    <hyperlink ref="K20" r:id="rId56"/>
-    <hyperlink ref="L20" r:id="rId57"/>
-    <hyperlink ref="J21" r:id="rId58"/>
-    <hyperlink ref="K21" r:id="rId59"/>
-    <hyperlink ref="L21" r:id="rId60"/>
-    <hyperlink ref="J22" r:id="rId61"/>
-    <hyperlink ref="K22" r:id="rId62"/>
-    <hyperlink ref="L22" r:id="rId63"/>
-    <hyperlink ref="J23" r:id="rId64"/>
-    <hyperlink ref="K23" r:id="rId65"/>
-    <hyperlink ref="L23" r:id="rId66"/>
-    <hyperlink ref="J24" r:id="rId67"/>
-    <hyperlink ref="K24" r:id="rId68"/>
-    <hyperlink ref="L24" r:id="rId69"/>
-    <hyperlink ref="J25" r:id="rId70"/>
-    <hyperlink ref="K25" r:id="rId71"/>
-    <hyperlink ref="L25" r:id="rId72"/>
-    <hyperlink ref="J26" r:id="rId73"/>
-    <hyperlink ref="K26" r:id="rId74"/>
-    <hyperlink ref="L26" r:id="rId75"/>
-    <hyperlink ref="J27" r:id="rId76"/>
-    <hyperlink ref="K27" r:id="rId77"/>
-    <hyperlink ref="L27" r:id="rId78"/>
-    <hyperlink ref="J28" r:id="rId79"/>
-    <hyperlink ref="K28" r:id="rId80"/>
-    <hyperlink ref="L28" r:id="rId81"/>
-    <hyperlink ref="J29" r:id="rId82"/>
-    <hyperlink ref="K29" r:id="rId83"/>
-    <hyperlink ref="L29" r:id="rId84"/>
-    <hyperlink ref="J30" r:id="rId85"/>
-    <hyperlink ref="K30" r:id="rId86"/>
-    <hyperlink ref="L30" r:id="rId87"/>
+    <hyperlink ref="M3" r:id="rId7"/>
+    <hyperlink ref="N3" r:id="rId8"/>
+    <hyperlink ref="J4" r:id="rId9"/>
+    <hyperlink ref="L4" r:id="rId10"/>
+    <hyperlink ref="M4" r:id="rId11"/>
+    <hyperlink ref="N4" r:id="rId12"/>
+    <hyperlink ref="J5" r:id="rId13"/>
+    <hyperlink ref="L5" r:id="rId14"/>
+    <hyperlink ref="M5" r:id="rId15"/>
+    <hyperlink ref="N5" r:id="rId16"/>
+    <hyperlink ref="J6" r:id="rId17"/>
+    <hyperlink ref="L6" r:id="rId18"/>
+    <hyperlink ref="M6" r:id="rId19"/>
+    <hyperlink ref="N6" r:id="rId20"/>
+    <hyperlink ref="J7" r:id="rId21"/>
+    <hyperlink ref="L7" r:id="rId22"/>
+    <hyperlink ref="M7" r:id="rId23"/>
+    <hyperlink ref="N7" r:id="rId24"/>
+    <hyperlink ref="L8" r:id="rId25"/>
+    <hyperlink ref="M8" r:id="rId26"/>
+    <hyperlink ref="N8" r:id="rId27"/>
+    <hyperlink ref="L9" r:id="rId28"/>
+    <hyperlink ref="M9" r:id="rId29"/>
+    <hyperlink ref="N9" r:id="rId30"/>
+    <hyperlink ref="J10" r:id="rId31"/>
+    <hyperlink ref="L10" r:id="rId32"/>
+    <hyperlink ref="M10" r:id="rId33"/>
+    <hyperlink ref="N10" r:id="rId34"/>
+    <hyperlink ref="L11" r:id="rId35"/>
+    <hyperlink ref="M11" r:id="rId36"/>
+    <hyperlink ref="N11" r:id="rId37"/>
+    <hyperlink ref="L12" r:id="rId38"/>
+    <hyperlink ref="M12" r:id="rId39"/>
+    <hyperlink ref="N12" r:id="rId40"/>
+    <hyperlink ref="J13" r:id="rId41"/>
+    <hyperlink ref="L13" r:id="rId42"/>
+    <hyperlink ref="M13" r:id="rId43"/>
+    <hyperlink ref="N13" r:id="rId44"/>
+    <hyperlink ref="J14" r:id="rId45"/>
+    <hyperlink ref="L14" r:id="rId46"/>
+    <hyperlink ref="M14" r:id="rId47"/>
+    <hyperlink ref="N14" r:id="rId48"/>
+    <hyperlink ref="J15" r:id="rId49"/>
+    <hyperlink ref="L15" r:id="rId50"/>
+    <hyperlink ref="M15" r:id="rId51"/>
+    <hyperlink ref="N15" r:id="rId52"/>
+    <hyperlink ref="L16" r:id="rId53"/>
+    <hyperlink ref="M16" r:id="rId54"/>
+    <hyperlink ref="N16" r:id="rId55"/>
+    <hyperlink ref="L17" r:id="rId56"/>
+    <hyperlink ref="M17" r:id="rId57"/>
+    <hyperlink ref="N17" r:id="rId58"/>
+    <hyperlink ref="J18" r:id="rId59"/>
+    <hyperlink ref="L18" r:id="rId60"/>
+    <hyperlink ref="M18" r:id="rId61"/>
+    <hyperlink ref="N18" r:id="rId62"/>
+    <hyperlink ref="J19" r:id="rId63"/>
+    <hyperlink ref="L19" r:id="rId64"/>
+    <hyperlink ref="M19" r:id="rId65"/>
+    <hyperlink ref="N19" r:id="rId66"/>
+    <hyperlink ref="L20" r:id="rId67"/>
+    <hyperlink ref="M20" r:id="rId68"/>
+    <hyperlink ref="N20" r:id="rId69"/>
+    <hyperlink ref="J21" r:id="rId70"/>
+    <hyperlink ref="L21" r:id="rId71"/>
+    <hyperlink ref="M21" r:id="rId72"/>
+    <hyperlink ref="N21" r:id="rId73"/>
+    <hyperlink ref="J22" r:id="rId74"/>
+    <hyperlink ref="L22" r:id="rId75"/>
+    <hyperlink ref="M22" r:id="rId76"/>
+    <hyperlink ref="N22" r:id="rId77"/>
+    <hyperlink ref="J23" r:id="rId78"/>
+    <hyperlink ref="L23" r:id="rId79"/>
+    <hyperlink ref="M23" r:id="rId80"/>
+    <hyperlink ref="N23" r:id="rId81"/>
+    <hyperlink ref="J24" r:id="rId82"/>
+    <hyperlink ref="L24" r:id="rId83"/>
+    <hyperlink ref="M24" r:id="rId84"/>
+    <hyperlink ref="N24" r:id="rId85"/>
+    <hyperlink ref="J25" r:id="rId86"/>
+    <hyperlink ref="L25" r:id="rId87"/>
+    <hyperlink ref="M25" r:id="rId88"/>
+    <hyperlink ref="N25" r:id="rId89"/>
+    <hyperlink ref="J26" r:id="rId90"/>
+    <hyperlink ref="L26" r:id="rId91"/>
+    <hyperlink ref="M26" r:id="rId92"/>
+    <hyperlink ref="N26" r:id="rId93"/>
+    <hyperlink ref="J27" r:id="rId94"/>
+    <hyperlink ref="L27" r:id="rId95"/>
+    <hyperlink ref="M27" r:id="rId96"/>
+    <hyperlink ref="N27" r:id="rId97"/>
+    <hyperlink ref="L28" r:id="rId98"/>
+    <hyperlink ref="M28" r:id="rId99"/>
+    <hyperlink ref="N28" r:id="rId100"/>
+    <hyperlink ref="L29" r:id="rId101"/>
+    <hyperlink ref="M29" r:id="rId102"/>
+    <hyperlink ref="N29" r:id="rId103"/>
+    <hyperlink ref="L30" r:id="rId104"/>
+    <hyperlink ref="M30" r:id="rId105"/>
+    <hyperlink ref="N30" r:id="rId106"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2686,7 +2959,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" style="9" customWidth="1"/>
@@ -2695,23 +2968,23 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>184</v>
+        <v>206</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>185</v>
+        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>186</v>
+        <v>208</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>187</v>
+        <v>209</v>
       </c>
       <c r="B3" s="10">
         <v>29</v>
@@ -2719,74 +2992,82 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>188</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>189</v>
+        <v>211</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>190</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>191</v>
+        <v>213</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>192</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>193</v>
+        <v>215</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>194</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>8</v>
+        <v>217</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>196</v>
+        <v>10</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>197</v>
+        <v>219</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>198</v>
+        <v>220</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>199</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>200</v>
+        <v>222</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>201</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>202</v>
+        <v>224</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>203</v>
+        <v>225</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>